<commit_message>
Actualiza dashboard campaña abril
</commit_message>
<xml_diff>
--- a/pages/RENDIMIENTO_ABRIL.xlsx
+++ b/pages/RENDIMIENTO_ABRIL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://arquimed-my.sharepoint.com/personal/manuel_toledo_arquimed_cl/Documents/VETERINARIA ARQUIMED/CARPETA DE TRABAJO 2026/DASH CCH/Commercial_Command_Hub/pages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E2D21E3-150F-4476-87D2-B9D0F7FB6406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{6E2D21E3-150F-4476-87D2-B9D0F7FB6406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A19FD00-03A8-4612-9743-2DBC4DCCF817}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{06545CA7-A51B-47E4-B217-A08FF6E0E8DD}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>REAGENT KIT V-52</t>
   </si>
@@ -61,9 +61,6 @@
   </si>
   <si>
     <t>Contactos</t>
-  </si>
-  <si>
-    <t>Conversaciones</t>
   </si>
   <si>
     <t>En Cierre</t>
@@ -480,21 +477,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB6C0EF5-4ED9-4935-851D-4CB9F3029165}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.85546875" customWidth="1"/>
-    <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" customWidth="1"/>
+    <col min="6" max="6" width="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="30">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="30">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -502,19 +498,19 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -523,15 +519,12 @@
         <v>9</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
         <v>10</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" t="s">
-        <v>11</v>
       </c>
       <c r="B2">
         <v>200</v>
@@ -542,19 +535,22 @@
       <c r="D2">
         <v>137</v>
       </c>
-      <c r="F2" s="1">
+      <c r="E2" s="1">
         <v>29</v>
       </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
       <c r="H2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>17740000</v>
       </c>
       <c r="J2">
-        <v>15500000</v>
-      </c>
-      <c r="K2">
         <v>353483</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega tabla CRM operacional
</commit_message>
<xml_diff>
--- a/pages/RENDIMIENTO_ABRIL.xlsx
+++ b/pages/RENDIMIENTO_ABRIL.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://arquimed-my.sharepoint.com/personal/manuel_toledo_arquimed_cl/Documents/VETERINARIA ARQUIMED/CARPETA DE TRABAJO 2026/DASH CCH/Commercial_Command_Hub/pages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{6E2D21E3-150F-4476-87D2-B9D0F7FB6406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A19FD00-03A8-4612-9743-2DBC4DCCF817}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{6E2D21E3-150F-4476-87D2-B9D0F7FB6406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D71B08BB-401D-4E92-A0AE-DC9EF970080B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{06545CA7-A51B-47E4-B217-A08FF6E0E8DD}"/>
+    <workbookView xWindow="10140" yWindow="0" windowWidth="10455" windowHeight="10905" firstSheet="1" activeTab="2" xr2:uid="{06545CA7-A51B-47E4-B217-A08FF6E0E8DD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Datos KPI" sheetId="1" r:id="rId1"/>
+    <sheet name="Insights" sheetId="2" r:id="rId2"/>
+    <sheet name="Referencias_CRM" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,19 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
-  <si>
-    <t>REAGENT KIT V-52</t>
-  </si>
-  <si>
-    <t>DIFF</t>
-  </si>
-  <si>
-    <t>LH</t>
-  </si>
-  <si>
-    <t>DIL 5.5</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Campaña</t>
   </si>
@@ -86,6 +75,84 @@
   </si>
   <si>
     <t>Oportunidades CRM arquimed</t>
+  </si>
+  <si>
+    <t>Insight</t>
+  </si>
+  <si>
+    <t>La campaña generó 200 leads desde Meta y 129 leads registrados en BoldKnight.</t>
+  </si>
+  <si>
+    <t>Se consolidaron 137 contactos comerciales efectivos.</t>
+  </si>
+  <si>
+    <t>Se lograron 29 agendamientos, equivalentes a 21.2% sobre contactos.</t>
+  </si>
+  <si>
+    <t>Se generaron 6 oportunidades comerciales reales.</t>
+  </si>
+  <si>
+    <t>La campaña ya generó 1 venta cerrada por $17.740.000.</t>
+  </si>
+  <si>
+    <t>El ROAS actual es de 50.2x, con una inversión de $353.483.</t>
+  </si>
+  <si>
+    <t>Existen 2 oportunidades en cierre, por lo que el resultado final aún puede aumentar.</t>
+  </si>
+  <si>
+    <t>Las ventas perdidas por falta de financiamiento deben registrarse como demanda no capturada, no como falta de interés comercial.</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>OCC</t>
+  </si>
+  <si>
+    <t>Oportunidad CRM</t>
+  </si>
+  <si>
+    <t>Cotización</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Valor CLP</t>
+  </si>
+  <si>
+    <t>KAM</t>
+  </si>
+  <si>
+    <t>Observación</t>
+  </si>
+  <si>
+    <t>Mevetlab</t>
+  </si>
+  <si>
+    <t>Vetus E7</t>
+  </si>
+  <si>
+    <t>OCC-2026-018</t>
+  </si>
+  <si>
+    <t>OPP-001245</t>
+  </si>
+  <si>
+    <t>COT-8892</t>
+  </si>
+  <si>
+    <t>En cierre</t>
+  </si>
+  <si>
+    <t>Manuel Toledo</t>
+  </si>
+  <si>
+    <t>Pendiente leasing</t>
   </si>
 </sst>
 </file>
@@ -134,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -142,6 +209,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -492,39 +565,39 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="30">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>200</v>
@@ -561,77 +634,124 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA8CB197-D1DE-4382-8301-BAD2C269F861}">
-  <dimension ref="B5:K9"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="120" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:11">
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>175000</v>
-      </c>
-      <c r="G5">
-        <f>(E5*F5)</f>
-        <v>700000</v>
-      </c>
-      <c r="J5">
-        <f>700000</f>
-        <v>700000</v>
-      </c>
-      <c r="K5">
-        <f>(J5/4)</f>
-        <v>175000</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11">
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11">
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11">
-      <c r="D8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>350000</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11">
-      <c r="D9" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>350000</v>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C905FB3D-BD9B-47FC-92A9-D9B5240E170B}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9" ht="30">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="30">
+      <c r="A2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="5">
+        <v>15500000</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>